<commit_message>
Daily tables: add new hires of 21/10
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HsFNnGJRzg6EEfnut1VvMX
</commit_message>
<xml_diff>
--- a/loss-time/outputs/Nhap_lieu_05-10_den_21-10.xlsx
+++ b/loss-time/outputs/Nhap_lieu_05-10_den_21-10.xlsx
@@ -9050,7 +9050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H39"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -9808,17 +9808,17 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-07/10</t>
+          <t>Đào tạo công nhân mới</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -9827,34 +9827,30 @@
         </is>
       </c>
       <c r="E22" s="5" t="n">
-        <v>0.3125</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="H22" s="6" t="inlineStr">
-        <is>
-          <t>A2 ngày 12/12 - nhóm 07/10</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-07/10</t>
+          <t>Đào tạo công nhân mới</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Raw Cutting</t>
+          <t>Machining</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
@@ -9863,34 +9859,30 @@
         </is>
       </c>
       <c r="E23" s="5" t="n">
-        <v>0.3125</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F23" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G23" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="H23" s="6" t="inlineStr">
-        <is>
-          <t>A2 ngày 12/12 - nhóm 07/10</t>
-        </is>
-      </c>
+      <c r="H23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>P22</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-08/10</t>
+          <t>Đào tạo công nhân mới</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>Raw Cutting</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
@@ -9899,19 +9891,15 @@
         </is>
       </c>
       <c r="E24" s="5" t="n">
-        <v>0.3125</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="F24" s="5" t="n">
-        <v>0.5</v>
+        <v>0.6666666666666666</v>
       </c>
       <c r="G24" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H24" s="6" t="inlineStr">
-        <is>
-          <t>A2 ngày 11/12 - nhóm 08/10</t>
-        </is>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="H24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
@@ -9921,12 +9909,12 @@
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-08/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-07/10</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>Machining</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
@@ -9941,11 +9929,11 @@
         <v>0.5</v>
       </c>
       <c r="G25" s="3" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="H25" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 11/12 - nhóm 08/10</t>
+          <t>A2 ngày 12/12 - nhóm 07/10</t>
         </is>
       </c>
     </row>
@@ -9957,12 +9945,12 @@
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-09/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-07/10</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
@@ -9977,11 +9965,11 @@
         <v>0.5</v>
       </c>
       <c r="G26" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="H26" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 10/12 - nhóm 09/10</t>
+          <t>A2 ngày 12/12 - nhóm 07/10</t>
         </is>
       </c>
     </row>
@@ -9993,7 +9981,7 @@
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-09/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-08/10</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
@@ -10013,11 +10001,11 @@
         <v>0.5</v>
       </c>
       <c r="G27" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H27" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 10/12 - nhóm 09/10</t>
+          <t>A2 ngày 11/12 - nhóm 08/10</t>
         </is>
       </c>
     </row>
@@ -10029,12 +10017,12 @@
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-12/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-08/10</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Machining</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
@@ -10049,11 +10037,11 @@
         <v>0.5</v>
       </c>
       <c r="G28" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H28" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 8/12 - nhóm 12/10</t>
+          <t>A2 ngày 11/12 - nhóm 08/10</t>
         </is>
       </c>
     </row>
@@ -10065,12 +10053,12 @@
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-12/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-09/10</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>Raw Cutting</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
@@ -10085,11 +10073,11 @@
         <v>0.5</v>
       </c>
       <c r="G29" s="3" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="H29" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 8/12 - nhóm 12/10</t>
+          <t>A2 ngày 10/12 - nhóm 09/10</t>
         </is>
       </c>
     </row>
@@ -10101,12 +10089,12 @@
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-09/10</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
@@ -10125,7 +10113,7 @@
       </c>
       <c r="H30" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 7/12 - nhóm 13/10</t>
+          <t>A2 ngày 10/12 - nhóm 09/10</t>
         </is>
       </c>
     </row>
@@ -10137,12 +10125,12 @@
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-12/10</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>Raw Cutting</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
@@ -10157,11 +10145,11 @@
         <v>0.5</v>
       </c>
       <c r="G31" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H31" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 7/12 - nhóm 13/10</t>
+          <t>A2 ngày 8/12 - nhóm 12/10</t>
         </is>
       </c>
     </row>
@@ -10173,12 +10161,12 @@
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-12/10</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>Machining</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
@@ -10197,7 +10185,7 @@
       </c>
       <c r="H32" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 7/12 - nhóm 13/10</t>
+          <t>A2 ngày 8/12 - nhóm 12/10</t>
         </is>
       </c>
     </row>
@@ -10209,7 +10197,7 @@
       </c>
       <c r="B33" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-14/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
@@ -10229,11 +10217,11 @@
         <v>0.5</v>
       </c>
       <c r="G33" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H33" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 6/12 - nhóm 14/10</t>
+          <t>A2 ngày 7/12 - nhóm 13/10</t>
         </is>
       </c>
     </row>
@@ -10245,12 +10233,12 @@
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-15/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Raw Cutting</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
@@ -10269,7 +10257,7 @@
       </c>
       <c r="H34" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 5/12 - nhóm 15/10</t>
+          <t>A2 ngày 7/12 - nhóm 13/10</t>
         </is>
       </c>
     </row>
@@ -10281,12 +10269,12 @@
       </c>
       <c r="B35" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-16/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-13/10</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>Assembly</t>
+          <t>Machining</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
@@ -10305,7 +10293,7 @@
       </c>
       <c r="H35" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 4/12 - nhóm 16/10</t>
+          <t>A2 ngày 7/12 - nhóm 13/10</t>
         </is>
       </c>
     </row>
@@ -10317,7 +10305,7 @@
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-19/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-14/10</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
@@ -10337,11 +10325,11 @@
         <v>0.5</v>
       </c>
       <c r="G36" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H36" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 2/12 - nhóm 19/10</t>
+          <t>A2 ngày 6/12 - nhóm 14/10</t>
         </is>
       </c>
     </row>
@@ -10353,12 +10341,12 @@
       </c>
       <c r="B37" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-19/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-15/10</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>Machining</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
@@ -10373,11 +10361,11 @@
         <v>0.5</v>
       </c>
       <c r="G37" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H37" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 2/12 - nhóm 19/10</t>
+          <t>A2 ngày 5/12 - nhóm 15/10</t>
         </is>
       </c>
     </row>
@@ -10389,7 +10377,7 @@
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-20/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-16/10</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
@@ -10409,11 +10397,11 @@
         <v>0.5</v>
       </c>
       <c r="G38" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="H38" s="6" t="inlineStr">
         <is>
-          <t>A2 ngày 1/12 - nhóm 20/10</t>
+          <t>A2 ngày 4/12 - nhóm 16/10</t>
         </is>
       </c>
     </row>
@@ -10425,12 +10413,12 @@
       </c>
       <c r="B39" s="4" t="inlineStr">
         <is>
-          <t>HC mới- 50% hiệu suất- 2 tuần-20/10</t>
+          <t>HC mới- 50% hiệu suất- 2 tuần-19/10</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>Machining</t>
+          <t>Assembly</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
@@ -10448,6 +10436,114 @@
         <v>2</v>
       </c>
       <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>A2 ngày 2/12 - nhóm 19/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>HC mới- 50% hiệu suất- 2 tuần-19/10</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Machining</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>HR/ HSE</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F40" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H40" s="6" t="inlineStr">
+        <is>
+          <t>A2 ngày 2/12 - nhóm 19/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B41" s="4" t="inlineStr">
+        <is>
+          <t>HC mới- 50% hiệu suất- 2 tuần-20/10</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>Assembly</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>HR/ HSE</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F41" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G41" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>A2 ngày 1/12 - nhóm 20/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>HC mới- 50% hiệu suất- 2 tuần-20/10</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Machining</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>HR/ HSE</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="F42" s="5" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="G42" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H42" s="6" t="inlineStr">
         <is>
           <t>A2 ngày 1/12 - nhóm 20/10</t>
         </is>

</xml_diff>